<commit_message>
Add editor background tools and Instagram roadmap
</commit_message>
<xml_diff>
--- a/outputs/pro_roadmap/Rubika_Publisher_Professional_Webapp_Roadmap_RFP_Backlog.xlsx
+++ b/outputs/pro_roadmap/Rubika_Publisher_Professional_Webapp_Roadmap_RFP_Backlog.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exec Summary" sheetId="1" r:id="Rfa1abdb84abb4a6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark" sheetId="2" r:id="R34b6d1593a534ca3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Audit" sheetId="3" r:id="R00325cd5ccd34b64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Phase Roadmap" sheetId="4" r:id="R5afcaeb440b94073"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFP Requirements" sheetId="5" r:id="Rf17a1e003eb04263"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="6" r:id="R81127e2fbe124e81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI UX System" sheetId="7" r:id="Rc93c224ceb554953"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Direction" sheetId="8" r:id="Rc4993895efb1499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Journeys" sheetId="9" r:id="Rb97f4e1f5b8d4ed8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="10" r:id="Ra7cead75029b42a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release KPI" sheetId="11" r:id="Rbaf3e5842a4643cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="12" r:id="Ra8da294fb9f3480c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exec Summary" sheetId="1" r:id="R9f70aee9685a4698"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark" sheetId="2" r:id="R5eb9e97ed99243ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Audit" sheetId="3" r:id="R47102b560c0348d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Phase Roadmap" sheetId="4" r:id="Re450de157ff34631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFP Requirements" sheetId="5" r:id="R3cdd2b65486b4020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="6" r:id="Ra7eb1d6911d94734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI UX System" sheetId="7" r:id="Rec8e65e7f120420b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theme Direction" sheetId="8" r:id="Rc827616724574fe2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Journeys" sheetId="9" r:id="R79df8adcdbde43fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="10" r:id="R59f413bc9d28443e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release KPI" sheetId="11" r:id="Rc52f1ed359f64c69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="12" r:id="R24c03912397a4641"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -119,48 +119,15 @@
   </x:fills>
   <x:borders count="10">
     <x:border/>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -382,7 +349,7 @@
         <x:color rgb="FFC24150"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1F2"/>
         </x:patternFill>
       </x:fill>
@@ -393,7 +360,7 @@
         <x:color rgb="FFB7791F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -404,7 +371,7 @@
         <x:color rgb="FF2563EB"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FF"/>
         </x:patternFill>
       </x:fill>
@@ -415,7 +382,7 @@
         <x:color rgb="FFC24150"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1F2"/>
         </x:patternFill>
       </x:fill>
@@ -426,7 +393,7 @@
         <x:color rgb="FFB7791F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -437,7 +404,7 @@
         <x:color rgb="FF2563EB"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FF"/>
         </x:patternFill>
       </x:fill>
@@ -627,7 +594,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R32a868b169a04ed0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcc43ec229ff443f9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1584,10 +1551,10 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbd4999fdbed4d0c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R299f5b90d86d4215"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41bdd5566baf43fe"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra486eb10511b4b76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b149fdeac9444d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2652eb4e581849ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1863,7 +1830,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5e9e687bd6644b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ea8653932cd4408"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2078,7 +2045,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc28f6e416954b34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9344edf1b738485a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2313,6 +2280,17 @@
         <x:v>Adjust release timing based on capacity.</x:v>
       </x:c>
     </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>Meta Instagram Platform Content Publishing</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>https://developers.facebook.com/docs/instagram-platform/content-publishing/</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Official reference for Instagram Graph API content publishing flow; re-check at implementation time.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -2320,8 +2298,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61af175e6d984f3c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36156c944c9d491f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c589f49df1e452a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref9848572f6c4243"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2495,7 +2473,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R309c93ca75e247ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73c087b7cb6e4905"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2727,7 +2705,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a925e059f384b54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6ab4c7af5a446bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3038,6 +3016,29 @@
         <x:v>Reports explain what worked, why, and what to do next</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Instagram Publishing Channel</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Meta OAuth, Instagram account connection, content publishing containers, queue worker, platform validation, channel analytics</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>Backend, frontend, devops</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Instagram professional account can connect, schedule, publish, retry, audit, and report alongside Rubika</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -3050,7 +3051,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R168e3b901b704820"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fe32466b26c4177"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3829,6 +3830,74 @@
         <x:v>Design</x:v>
       </x:c>
     </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>FR-044</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>Instagram account connection</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>Workspace can connect, validate, disconnect, and reconnect an Instagram professional account through Meta OAuth.</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>Publishing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>FR-045</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>Instagram content publishing</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>System creates Instagram media containers, publishes them through a durable worker, and records external ids/permalinks.</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>Publishing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>FR-046</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>Multi-channel composer</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Composer supports Rubika, Instagram, or both with platform-specific validation before scheduling.</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>Composer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>NFR-012</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>Credential security</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>Instagram access tokens are encrypted, scoped, refresh-aware, and never exposed in logs or UI.</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -3836,7 +3905,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e8dcf8ae8b3428f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a75e5a9eb834c03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5528,6 +5597,122 @@
         <x:v>New engineer can run app and tests</x:v>
       </x:c>
     </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>B-057</x:v>
+      </x:c>
+      <x:c r="B61" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>Instagram Connection</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>Create Meta OAuth connection flow and Instagram account model</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F61" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>Publishing Reliability</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>Use Meta app OAuth, store encrypted tokens, account/page identifiers, expiry, reconnect and disconnect flows</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>Workspace can connect and validate an Instagram professional account</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>B-058</x:v>
+      </x:c>
+      <x:c r="B62" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>Instagram Publishing</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>Publish scheduled posts to Instagram through worker jobs</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F62" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>B-057, worker reliability</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>Create media container, poll readiness when needed, publish container, store external id/permalink, classify errors</x:v>
+      </x:c>
+      <x:c r="I62" t="str">
+        <x:v>Scheduled Instagram post publishes once with auditable job state</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>B-059</x:v>
+      </x:c>
+      <x:c r="B63" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>Platform Validation</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>Add Instagram validation to composer and media editor</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F63" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>Media DAM Pro, Composer Studio Pro</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>Validate format, aspect ratio, file type, caption, channel selection, and export readiness before scheduling</x:v>
+      </x:c>
+      <x:c r="I63" t="str">
+        <x:v>Invalid Instagram posts are blocked before queueing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>B-060</x:v>
+      </x:c>
+      <x:c r="B64" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>Channel Analytics</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>Add Instagram channel filters and published id metrics</x:v>
+      </x:c>
+      <x:c r="E64" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F64" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>Analytics events</x:v>
+      </x:c>
+      <x:c r="H64" t="str">
+        <x:v>Capture published id/permalink and channel-specific event metadata for reports and filters</x:v>
+      </x:c>
+      <x:c r="I64" t="str">
+        <x:v>Content, queue, logs, calendar, and analytics can filter Instagram posts</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -5540,7 +5725,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re10e37b8dff94215"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4a72ebf218d4184"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5744,7 +5929,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ce9229609e041db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8eaf02862c0647cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5976,7 +6161,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbca8c2c89bf44f47"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4249a9b0b27e47e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6184,7 +6369,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2bdaf72e8849a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9de78808ee4d46c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>